<commit_message>
Update soccer trades 2026-07-30 09:01:46 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Primera A/trades.xlsx
+++ b/data/sxbet/ligas/Primera A/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V3"/>
+  <dimension ref="A1:V4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,102 +531,94 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0x9ff1fda59e1de553a293f3669eef33f243c577ad387b1abf6cbe9347473b44c6</t>
+          <t>0x7329421797dc603c2125293bb4d7a5bfcff5a6ef4e85c5df6823893cb97e17ee</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>60.05998</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>1.7575</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Primera A</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>CDP Junior FC vs Millonarios</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>CDP Junior FC</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Millonarios</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>0x0793e576da59b70aa8ea4c5fb634c02f46858b912ecd6a02f91f6ebbaa986be7</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>L19606649</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>1.6637</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Atlético Bucaramanga</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Primera A</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Atlético Bucaramanga vs Llaneros FC</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>Atlético Bucaramanga</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Llaneros FC</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>0x0a67b48214c191d8392e1d2d3f46113bbde830da36a1ff74ffb1f181c08e506b</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>L19614187</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>SUCCESS</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1785344668</t>
+          <t>1785400533</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1785459600</t>
+          <t>1785633300</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>1.506591</t>
+          <t>79.287102</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -643,110 +635,222 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>0x9ff1fda59e1de553a293f3669eef33f243c577ad387b1abf6cbe9347473b44c6</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>1.6637</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Atlético Bucaramanga</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Primera A</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Atlético Bucaramanga vs Llaneros FC</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Atlético Bucaramanga</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Llaneros FC</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>0x0a67b48214c191d8392e1d2d3f46113bbde830da36a1ff74ffb1f181c08e506b</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>L19614187</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>1785344668</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>1785459600</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>1.506591</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
           <t>0xb99da8b648376c357d13a6060e6f4dc2ae7491c558b543e4c668392cdfe2e5bd</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>0.99999</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>1.6987</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>1X2</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>Fortaleza CEIF</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>Primera A</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>Fortaleza CEIF vs Deportivo Pereira</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>Fortaleza CEIF</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>Deportivo Pereira</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>0xd09cb30bf0c8317660cdcbbfc8ea542253305047aabd0fa7acee0ff117d36274</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>L19596272</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
+      <c r="P4" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr">
+      <c r="Q4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr">
+      <c r="R4" t="inlineStr">
         <is>
           <t>1785344544</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr">
+      <c r="S4" t="inlineStr">
         <is>
           <t>1785546000</t>
         </is>
       </c>
-      <c r="T3" t="inlineStr">
+      <c r="T4" t="inlineStr">
         <is>
           <t>1.431113</t>
         </is>
       </c>
-      <c r="U3" t="inlineStr">
+      <c r="U4" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V3" t="inlineStr">
+      <c r="V4" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-07-30 19:03:06 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Primera A/trades.xlsx
+++ b/data/sxbet/ligas/Primera A/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V4"/>
+  <dimension ref="A1:V5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,28 +531,28 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0x7329421797dc603c2125293bb4d7a5bfcff5a6ef4e85c5df6823893cb97e17ee</t>
+          <t>0x407971887685061312685cb0b7f5ef9ed6261d2f1b2d1f09c45aa4eae0a05e25</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>60.05998</t>
+          <t>3.57999</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.7575</t>
+          <t>1.5425</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
@@ -563,27 +563,27 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>CDP Junior FC vs Millonarios</t>
+          <t>Atlético Bucaramanga vs Llaneros FC</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>CDP Junior FC</t>
+          <t>Atlético Bucaramanga</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Millonarios</t>
+          <t>Llaneros FC</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0x0793e576da59b70aa8ea4c5fb634c02f46858b912ecd6a02f91f6ebbaa986be7</t>
+          <t>0x481fdaa2a20c002d515f3c43eac07f52063302592153594bc8cb3d995852a008</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>L19606649</t>
+          <t>L19614187</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -608,17 +608,17 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1785400533</t>
+          <t>1785434777</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1785633300</t>
+          <t>1785459600</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>79.287102</t>
+          <t>6.59906</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -635,102 +635,94 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0x9ff1fda59e1de553a293f3669eef33f243c577ad387b1abf6cbe9347473b44c6</t>
+          <t>0x7329421797dc603c2125293bb4d7a5bfcff5a6ef4e85c5df6823893cb97e17ee</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>60.05998</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>1.7575</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Primera A</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>CDP Junior FC vs Millonarios</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>CDP Junior FC</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Millonarios</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>0x0793e576da59b70aa8ea4c5fb634c02f46858b912ecd6a02f91f6ebbaa986be7</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>L19606649</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>1.6637</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Atlético Bucaramanga</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Primera A</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>Atlético Bucaramanga vs Llaneros FC</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>Atlético Bucaramanga</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Llaneros FC</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>0x0a67b48214c191d8392e1d2d3f46113bbde830da36a1ff74ffb1f181c08e506b</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>L19614187</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>SUCCESS</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1785344668</t>
+          <t>1785400533</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>1785459600</t>
+          <t>1785633300</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>1.506591</t>
+          <t>79.287102</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -747,110 +739,222 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>0x9ff1fda59e1de553a293f3669eef33f243c577ad387b1abf6cbe9347473b44c6</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>1.6637</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Atlético Bucaramanga</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Primera A</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Atlético Bucaramanga vs Llaneros FC</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Atlético Bucaramanga</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Llaneros FC</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>0x0a67b48214c191d8392e1d2d3f46113bbde830da36a1ff74ffb1f181c08e506b</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>L19614187</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>1785344668</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>1785459600</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>1.506591</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
           <t>0xb99da8b648376c357d13a6060e6f4dc2ae7491c558b543e4c668392cdfe2e5bd</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>0.99999</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>1.6987</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>1X2</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>Fortaleza CEIF</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>Primera A</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>Fortaleza CEIF vs Deportivo Pereira</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>Fortaleza CEIF</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>Deportivo Pereira</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>0xd09cb30bf0c8317660cdcbbfc8ea542253305047aabd0fa7acee0ff117d36274</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>L19596272</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr">
+      <c r="O5" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="P5" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr">
+      <c r="Q5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="R4" t="inlineStr">
+      <c r="R5" t="inlineStr">
         <is>
           <t>1785344544</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr">
+      <c r="S5" t="inlineStr">
         <is>
           <t>1785546000</t>
         </is>
       </c>
-      <c r="T4" t="inlineStr">
+      <c r="T5" t="inlineStr">
         <is>
           <t>1.431113</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr">
+      <c r="U5" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V4" t="inlineStr">
+      <c r="V5" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>